<commit_message>
feat: verify rule CG0395 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000130/negative/01/data/unit-test-coreid-CG0395-negative.xlsx
+++ b/rules/CORE-000130/negative/01/data/unit-test-coreid-CG0395-negative.xlsx
@@ -35,7 +35,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +46,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -104,6 +110,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -545,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -577,6 +587,62 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AESMIE</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AESMIE</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>MAYBE</t>
         </is>
       </c>
     </row>
@@ -591,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y5"/>
+  <dimension ref="A1:Y8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1136,7 +1202,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="R5" s="5" t="inlineStr">
+      <c r="R5" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -1164,6 +1230,336 @@
       </c>
       <c r="X5" s="5" t="n"/>
       <c r="Y5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CDISC009</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>HEADACHE</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>MILD</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>DOSE NOT CHANGED</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>POSSIBLY RELATED</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>RECOVERED/RESOLVED</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R6" s="7" t="inlineStr">
+        <is>
+          <t>MAYBE</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>TREATMENT</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>2014-11-15</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>2014-11-20</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>180</v>
+      </c>
+      <c r="W6" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CDISC010</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NAUSEA</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>MODERATE</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>DOSE NOT CHANGED</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>RELATED</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>NOT RECOVERED/NOT RESOLVED</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>TREATMENT</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>2014-12-01</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>196</v>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>ONGOING</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>2015-01-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CDISC011</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DIZZINESS</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>MILD</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>DOSE NOT CHANGED</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>NOT RELATED</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>RECOVERED/RESOLVED</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>TREATMENT</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>2014-12-10</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>2014-12-12</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>205</v>
+      </c>
+      <c r="W8" t="n">
+        <v>207</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>